<commit_message>
Add Data Model Draft
</commit_message>
<xml_diff>
--- a/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
+++ b/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
@@ -211,37 +211,37 @@
     <t>Medium</t>
   </si>
   <si>
+    <t>docs/sprints/S0.3.md</t>
+  </si>
+  <si>
+    <t>Naming standards published</t>
+  </si>
+  <si>
+    <t>S0.4</t>
+  </si>
+  <si>
+    <t>Define Data Models</t>
+  </si>
+  <si>
+    <t>Data Model Draft</t>
+  </si>
+  <si>
+    <t>docs/sprints/S0.4.md</t>
+  </si>
+  <si>
+    <t>Core data models documented</t>
+  </si>
+  <si>
+    <t>S0.5</t>
+  </si>
+  <si>
+    <t>Define Bronze Silver Gold Strategy</t>
+  </si>
+  <si>
+    <t>Data Layer Design</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>docs/sprints/S0.3.md</t>
-  </si>
-  <si>
-    <t>Naming standards published</t>
-  </si>
-  <si>
-    <t>S0.4</t>
-  </si>
-  <si>
-    <t>Define Data Models</t>
-  </si>
-  <si>
-    <t>Data Model Draft</t>
-  </si>
-  <si>
-    <t>docs/sprints/S0.4.md</t>
-  </si>
-  <si>
-    <t>Core data models documented</t>
-  </si>
-  <si>
-    <t>S0.5</t>
-  </si>
-  <si>
-    <t>Define Bronze Silver Gold Strategy</t>
-  </si>
-  <si>
-    <t>Data Layer Design</t>
   </si>
   <si>
     <t>docs/sprints/S0.5.md</t>
@@ -1533,16 +1533,16 @@
         <v>63</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="G4" s="5">
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>55</v>
@@ -1554,28 +1554,28 @@
         <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="G5" s="5">
         <v>2</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>48</v>
@@ -1587,19 +1587,19 @@
         <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G6" s="5">
         <v>2</v>
@@ -1632,7 +1632,7 @@
         <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G7" s="5">
         <v>1</v>
@@ -1644,7 +1644,7 @@
         <v>82</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7" s="1"/>
     </row>
@@ -1665,7 +1665,7 @@
         <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G8" s="5">
         <v>2</v>
@@ -1698,7 +1698,7 @@
         <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
@@ -1731,7 +1731,7 @@
         <v>51</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G10" s="5">
         <v>2</v>
@@ -1764,7 +1764,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G11" s="5">
         <v>2</v>
@@ -1797,7 +1797,7 @@
         <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G12" s="5">
         <v>2</v>
@@ -1830,7 +1830,7 @@
         <v>63</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G13" s="5">
         <v>2</v>
@@ -1863,7 +1863,7 @@
         <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G14" s="5">
         <v>2</v>
@@ -1896,7 +1896,7 @@
         <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G15" s="5">
         <v>2</v>
@@ -1929,7 +1929,7 @@
         <v>51</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G16" s="5">
         <v>2</v>
@@ -1962,7 +1962,7 @@
         <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G17" s="5">
         <v>2</v>
@@ -1995,7 +1995,7 @@
         <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G18" s="5">
         <v>2</v>
@@ -2028,7 +2028,7 @@
         <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G19" s="5">
         <v>2</v>
@@ -2061,7 +2061,7 @@
         <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G20" s="5">
         <v>2</v>
@@ -2094,7 +2094,7 @@
         <v>63</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G21" s="5">
         <v>2</v>
@@ -2127,7 +2127,7 @@
         <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G22" s="5">
         <v>2</v>
@@ -2160,7 +2160,7 @@
         <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G23" s="5">
         <v>2</v>
@@ -2193,7 +2193,7 @@
         <v>63</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
@@ -2226,7 +2226,7 @@
         <v>174</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G25" s="5">
         <v>2</v>
@@ -2259,7 +2259,7 @@
         <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
@@ -2292,7 +2292,7 @@
         <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
@@ -2325,7 +2325,7 @@
         <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
@@ -2358,7 +2358,7 @@
         <v>63</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G29" s="5">
         <v>2</v>
@@ -2391,7 +2391,7 @@
         <v>63</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G30" s="5">
         <v>2</v>
@@ -2424,7 +2424,7 @@
         <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G31" s="5">
         <v>2</v>
@@ -2457,7 +2457,7 @@
         <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G32" s="5">
         <v>2</v>
@@ -2490,7 +2490,7 @@
         <v>63</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G33" s="5">
         <v>2</v>
@@ -2523,7 +2523,7 @@
         <v>63</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G34" s="5">
         <v>2</v>
@@ -2556,7 +2556,7 @@
         <v>174</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>63</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G36" s="5">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         <v>63</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G37" s="5">
         <v>2</v>
@@ -2655,7 +2655,7 @@
         <v>63</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G38" s="5">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>174</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G39" s="5">
         <v>2</v>
@@ -2721,7 +2721,7 @@
         <v>174</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
@@ -2754,7 +2754,7 @@
         <v>63</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G41" s="5">
         <v>2</v>
@@ -2787,7 +2787,7 @@
         <v>174</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G42" s="5">
         <v>2</v>
@@ -2820,7 +2820,7 @@
         <v>63</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G43" s="5">
         <v>2</v>
@@ -2853,7 +2853,7 @@
         <v>63</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G44" s="5">
         <v>2</v>
@@ -2886,7 +2886,7 @@
         <v>63</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G45" s="5">
         <v>2</v>
@@ -2919,7 +2919,7 @@
         <v>63</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G46" s="5">
         <v>2</v>
@@ -2952,7 +2952,7 @@
         <v>174</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G47" s="5">
         <v>2</v>
@@ -2985,7 +2985,7 @@
         <v>174</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G48" s="5">
         <v>2</v>
@@ -3018,7 +3018,7 @@
         <v>174</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G49" s="5">
         <v>2</v>
@@ -3051,7 +3051,7 @@
         <v>174</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G50" s="5">
         <v>2</v>
@@ -3084,7 +3084,7 @@
         <v>174</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G51" s="5">
         <v>2</v>
@@ -3117,7 +3117,7 @@
         <v>174</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G52" s="5">
         <v>2</v>

</xml_diff>

<commit_message>
Add Define Bronze Silver Gold Strategy
</commit_message>
<xml_diff>
--- a/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
+++ b/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
@@ -241,25 +241,25 @@
     <t>Data Layer Design</t>
   </si>
   <si>
+    <t>docs/sprints/S0.5.md</t>
+  </si>
+  <si>
+    <t>Medallion architecture documented</t>
+  </si>
+  <si>
+    <t>S0.2,S0.4</t>
+  </si>
+  <si>
+    <t>S0.6</t>
+  </si>
+  <si>
+    <t>Define Physical Data Layout</t>
+  </si>
+  <si>
+    <t>Catalog / Schema / Dataset Structure</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>docs/sprints/S0.5.md</t>
-  </si>
-  <si>
-    <t>Medallion architecture documented</t>
-  </si>
-  <si>
-    <t>S0.2,S0.4</t>
-  </si>
-  <si>
-    <t>S0.6</t>
-  </si>
-  <si>
-    <t>Define Physical Data Layout</t>
-  </si>
-  <si>
-    <t>Catalog / Schema / Dataset Structure</t>
   </si>
   <si>
     <t>docs/sprints/S0.6.md</t>
@@ -1599,19 +1599,19 @@
         <v>51</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="5">
+        <v>2</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="5">
-        <v>2</v>
-      </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="K6" s="1"/>
     </row>
@@ -1620,19 +1620,19 @@
         <v>47</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G7" s="5">
         <v>1</v>
@@ -1665,7 +1665,7 @@
         <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G8" s="5">
         <v>2</v>
@@ -1698,7 +1698,7 @@
         <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
@@ -1731,7 +1731,7 @@
         <v>51</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G10" s="5">
         <v>2</v>
@@ -1764,7 +1764,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G11" s="5">
         <v>2</v>
@@ -1797,7 +1797,7 @@
         <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G12" s="5">
         <v>2</v>
@@ -1830,7 +1830,7 @@
         <v>63</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G13" s="5">
         <v>2</v>
@@ -1863,7 +1863,7 @@
         <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G14" s="5">
         <v>2</v>
@@ -1896,7 +1896,7 @@
         <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G15" s="5">
         <v>2</v>
@@ -1929,7 +1929,7 @@
         <v>51</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G16" s="5">
         <v>2</v>
@@ -1962,7 +1962,7 @@
         <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G17" s="5">
         <v>2</v>
@@ -1995,7 +1995,7 @@
         <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G18" s="5">
         <v>2</v>
@@ -2028,7 +2028,7 @@
         <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G19" s="5">
         <v>2</v>
@@ -2061,7 +2061,7 @@
         <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G20" s="5">
         <v>2</v>
@@ -2094,7 +2094,7 @@
         <v>63</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G21" s="5">
         <v>2</v>
@@ -2127,7 +2127,7 @@
         <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G22" s="5">
         <v>2</v>
@@ -2160,7 +2160,7 @@
         <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G23" s="5">
         <v>2</v>
@@ -2193,7 +2193,7 @@
         <v>63</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
@@ -2226,7 +2226,7 @@
         <v>174</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G25" s="5">
         <v>2</v>
@@ -2259,7 +2259,7 @@
         <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
@@ -2292,7 +2292,7 @@
         <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
@@ -2325,7 +2325,7 @@
         <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
@@ -2358,7 +2358,7 @@
         <v>63</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G29" s="5">
         <v>2</v>
@@ -2391,7 +2391,7 @@
         <v>63</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G30" s="5">
         <v>2</v>
@@ -2424,7 +2424,7 @@
         <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G31" s="5">
         <v>2</v>
@@ -2457,7 +2457,7 @@
         <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G32" s="5">
         <v>2</v>
@@ -2490,7 +2490,7 @@
         <v>63</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G33" s="5">
         <v>2</v>
@@ -2523,7 +2523,7 @@
         <v>63</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G34" s="5">
         <v>2</v>
@@ -2556,7 +2556,7 @@
         <v>174</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>63</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G36" s="5">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         <v>63</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G37" s="5">
         <v>2</v>
@@ -2655,7 +2655,7 @@
         <v>63</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G38" s="5">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>174</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G39" s="5">
         <v>2</v>
@@ -2721,7 +2721,7 @@
         <v>174</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
@@ -2754,7 +2754,7 @@
         <v>63</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G41" s="5">
         <v>2</v>
@@ -2787,7 +2787,7 @@
         <v>174</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G42" s="5">
         <v>2</v>
@@ -2820,7 +2820,7 @@
         <v>63</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G43" s="5">
         <v>2</v>
@@ -2853,7 +2853,7 @@
         <v>63</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G44" s="5">
         <v>2</v>
@@ -2886,7 +2886,7 @@
         <v>63</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G45" s="5">
         <v>2</v>
@@ -2919,7 +2919,7 @@
         <v>63</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G46" s="5">
         <v>2</v>
@@ -2952,7 +2952,7 @@
         <v>174</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G47" s="5">
         <v>2</v>
@@ -2985,7 +2985,7 @@
         <v>174</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G48" s="5">
         <v>2</v>
@@ -3018,7 +3018,7 @@
         <v>174</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G49" s="5">
         <v>2</v>
@@ -3051,7 +3051,7 @@
         <v>174</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G50" s="5">
         <v>2</v>
@@ -3084,7 +3084,7 @@
         <v>174</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G51" s="5">
         <v>2</v>
@@ -3117,7 +3117,7 @@
         <v>174</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G52" s="5">
         <v>2</v>

</xml_diff>

<commit_message>
Add Define Physical Data Layout
</commit_message>
<xml_diff>
--- a/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
+++ b/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
@@ -178,7 +178,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>docs/sprints/S0.1.md</t>
+    <t>docs/project_scope.md</t>
   </si>
   <si>
     <t>Project scope documented</t>
@@ -193,7 +193,7 @@
     <t>Repository Structure</t>
   </si>
   <si>
-    <t>docs/sprints/S0.2.md</t>
+    <t>docs/architecture/architecture_decisions.md</t>
   </si>
   <si>
     <t>Folder structure approved</t>
@@ -211,7 +211,7 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>docs/sprints/S0.3.md</t>
+    <t>docs/naming_conventions.md</t>
   </si>
   <si>
     <t>Naming standards published</t>
@@ -226,7 +226,7 @@
     <t>Data Model Draft</t>
   </si>
   <si>
-    <t>docs/sprints/S0.4.md</t>
+    <t>docs/data_models.md</t>
   </si>
   <si>
     <t>Core data models documented</t>
@@ -241,7 +241,7 @@
     <t>Data Layer Design</t>
   </si>
   <si>
-    <t>docs/sprints/S0.5.md</t>
+    <t>docs/lakehouse_architecture.md</t>
   </si>
   <si>
     <t>Medallion architecture documented</t>
@@ -259,25 +259,25 @@
     <t>Catalog / Schema / Dataset Structure</t>
   </si>
   <si>
+    <t>docs/physical_data_layout.md</t>
+  </si>
+  <si>
+    <t>Physical layout approved</t>
+  </si>
+  <si>
+    <t>Strava Ingestion</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>Create Strava Application</t>
+  </si>
+  <si>
+    <t>Client ID and Client Secret</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>docs/sprints/S0.6.md</t>
-  </si>
-  <si>
-    <t>Physical layout approved</t>
-  </si>
-  <si>
-    <t>Strava Ingestion</t>
-  </si>
-  <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>Create Strava Application</t>
-  </si>
-  <si>
-    <t>Client ID and Client Secret</t>
   </si>
   <si>
     <t>docs/sprints/S1.md</t>
@@ -1411,7 +1411,7 @@
     <col min="5" max="5" style="2" width="11.005" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="2" width="14.005" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="6" width="23.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="2" width="23.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="2" width="28.862142857142857" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="2" width="51.005" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="2" width="15.005" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="2" width="8.005" customWidth="1" bestFit="1"/>
@@ -1632,16 +1632,16 @@
         <v>51</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="G7" s="5">
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>71</v>
@@ -1650,22 +1650,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G8" s="5">
         <v>2</v>
@@ -1683,7 +1683,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>89</v>
@@ -1698,7 +1698,7 @@
         <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
@@ -1710,13 +1710,13 @@
         <v>93</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>94</v>
@@ -1731,7 +1731,7 @@
         <v>51</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G10" s="5">
         <v>2</v>
@@ -1749,7 +1749,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>99</v>
@@ -1764,7 +1764,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G11" s="5">
         <v>2</v>
@@ -1782,7 +1782,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>105</v>
@@ -1797,7 +1797,7 @@
         <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G12" s="5">
         <v>2</v>
@@ -1815,7 +1815,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>110</v>
@@ -1830,7 +1830,7 @@
         <v>63</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G13" s="5">
         <v>2</v>
@@ -1848,7 +1848,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>115</v>
@@ -1863,7 +1863,7 @@
         <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G14" s="5">
         <v>2</v>
@@ -1881,7 +1881,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>120</v>
@@ -1896,7 +1896,7 @@
         <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G15" s="5">
         <v>2</v>
@@ -1929,7 +1929,7 @@
         <v>51</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G16" s="5">
         <v>2</v>
@@ -1962,7 +1962,7 @@
         <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G17" s="5">
         <v>2</v>
@@ -1995,7 +1995,7 @@
         <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G18" s="5">
         <v>2</v>
@@ -2028,7 +2028,7 @@
         <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G19" s="5">
         <v>2</v>
@@ -2061,7 +2061,7 @@
         <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G20" s="5">
         <v>2</v>
@@ -2094,7 +2094,7 @@
         <v>63</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G21" s="5">
         <v>2</v>
@@ -2127,7 +2127,7 @@
         <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G22" s="5">
         <v>2</v>
@@ -2160,7 +2160,7 @@
         <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G23" s="5">
         <v>2</v>
@@ -2193,7 +2193,7 @@
         <v>63</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
@@ -2226,7 +2226,7 @@
         <v>174</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G25" s="5">
         <v>2</v>
@@ -2259,7 +2259,7 @@
         <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
@@ -2292,7 +2292,7 @@
         <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
@@ -2325,7 +2325,7 @@
         <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
@@ -2358,7 +2358,7 @@
         <v>63</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G29" s="5">
         <v>2</v>
@@ -2391,7 +2391,7 @@
         <v>63</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G30" s="5">
         <v>2</v>
@@ -2424,7 +2424,7 @@
         <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G31" s="5">
         <v>2</v>
@@ -2457,7 +2457,7 @@
         <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G32" s="5">
         <v>2</v>
@@ -2490,7 +2490,7 @@
         <v>63</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G33" s="5">
         <v>2</v>
@@ -2523,7 +2523,7 @@
         <v>63</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G34" s="5">
         <v>2</v>
@@ -2556,7 +2556,7 @@
         <v>174</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>63</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G36" s="5">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         <v>63</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G37" s="5">
         <v>2</v>
@@ -2655,7 +2655,7 @@
         <v>63</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G38" s="5">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>174</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G39" s="5">
         <v>2</v>
@@ -2721,7 +2721,7 @@
         <v>174</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
@@ -2754,7 +2754,7 @@
         <v>63</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G41" s="5">
         <v>2</v>
@@ -2787,7 +2787,7 @@
         <v>174</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G42" s="5">
         <v>2</v>
@@ -2820,7 +2820,7 @@
         <v>63</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G43" s="5">
         <v>2</v>
@@ -2853,7 +2853,7 @@
         <v>63</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G44" s="5">
         <v>2</v>
@@ -2886,7 +2886,7 @@
         <v>63</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G45" s="5">
         <v>2</v>
@@ -2919,7 +2919,7 @@
         <v>63</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G46" s="5">
         <v>2</v>
@@ -2952,7 +2952,7 @@
         <v>174</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G47" s="5">
         <v>2</v>
@@ -2985,7 +2985,7 @@
         <v>174</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G48" s="5">
         <v>2</v>
@@ -3018,7 +3018,7 @@
         <v>174</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G49" s="5">
         <v>2</v>
@@ -3051,7 +3051,7 @@
         <v>174</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G50" s="5">
         <v>2</v>
@@ -3084,7 +3084,7 @@
         <v>174</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G51" s="5">
         <v>2</v>
@@ -3117,7 +3117,7 @@
         <v>174</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="G52" s="5">
         <v>2</v>

</xml_diff>

<commit_message>
Add Strava setup documentation
</commit_message>
<xml_diff>
--- a/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
+++ b/docs/roadmap/Fitness_Data_Platform_Roadmap_v5.xlsx
@@ -277,22 +277,22 @@
     <t>Client ID and Client Secret</t>
   </si>
   <si>
+    <t>docs/sprints/S1.md</t>
+  </si>
+  <si>
+    <t>Create Strava Application completed</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>Implement OAuth Authentication</t>
+  </si>
+  <si>
+    <t>Refresh Token</t>
+  </si>
+  <si>
     <t>Not Started</t>
-  </si>
-  <si>
-    <t>docs/sprints/S1.md</t>
-  </si>
-  <si>
-    <t>Create Strava Application completed</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>Implement OAuth Authentication</t>
-  </si>
-  <si>
-    <t>Refresh Token</t>
   </si>
   <si>
     <t>docs/sprints/S2.md</t>
@@ -1665,16 +1665,16 @@
         <v>51</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="5">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="5">
-        <v>2</v>
-      </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>48</v>
@@ -1686,19 +1686,19 @@
         <v>82</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>51</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
@@ -1731,7 +1731,7 @@
         <v>51</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G10" s="5">
         <v>2</v>
@@ -1743,7 +1743,7 @@
         <v>98</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K10" s="1"/>
     </row>
@@ -1764,7 +1764,7 @@
         <v>51</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G11" s="5">
         <v>2</v>
@@ -1797,7 +1797,7 @@
         <v>51</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G12" s="5">
         <v>2</v>
@@ -1830,7 +1830,7 @@
         <v>63</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G13" s="5">
         <v>2</v>
@@ -1863,7 +1863,7 @@
         <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G14" s="5">
         <v>2</v>
@@ -1896,7 +1896,7 @@
         <v>51</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G15" s="5">
         <v>2</v>
@@ -1929,7 +1929,7 @@
         <v>51</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G16" s="5">
         <v>2</v>
@@ -1962,7 +1962,7 @@
         <v>51</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G17" s="5">
         <v>2</v>
@@ -1995,7 +1995,7 @@
         <v>51</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G18" s="5">
         <v>2</v>
@@ -2028,7 +2028,7 @@
         <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G19" s="5">
         <v>2</v>
@@ -2061,7 +2061,7 @@
         <v>51</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G20" s="5">
         <v>2</v>
@@ -2094,7 +2094,7 @@
         <v>63</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G21" s="5">
         <v>2</v>
@@ -2127,7 +2127,7 @@
         <v>51</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G22" s="5">
         <v>2</v>
@@ -2160,7 +2160,7 @@
         <v>51</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G23" s="5">
         <v>2</v>
@@ -2193,7 +2193,7 @@
         <v>63</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
@@ -2226,7 +2226,7 @@
         <v>174</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G25" s="5">
         <v>2</v>
@@ -2259,7 +2259,7 @@
         <v>51</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
@@ -2292,7 +2292,7 @@
         <v>51</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
@@ -2325,7 +2325,7 @@
         <v>51</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
@@ -2358,7 +2358,7 @@
         <v>63</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G29" s="5">
         <v>2</v>
@@ -2391,7 +2391,7 @@
         <v>63</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G30" s="5">
         <v>2</v>
@@ -2424,7 +2424,7 @@
         <v>51</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G31" s="5">
         <v>2</v>
@@ -2457,7 +2457,7 @@
         <v>51</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G32" s="5">
         <v>2</v>
@@ -2490,7 +2490,7 @@
         <v>63</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G33" s="5">
         <v>2</v>
@@ -2523,7 +2523,7 @@
         <v>63</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G34" s="5">
         <v>2</v>
@@ -2556,7 +2556,7 @@
         <v>174</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
@@ -2589,7 +2589,7 @@
         <v>63</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G36" s="5">
         <v>2</v>
@@ -2622,7 +2622,7 @@
         <v>63</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G37" s="5">
         <v>2</v>
@@ -2655,7 +2655,7 @@
         <v>63</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G38" s="5">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>174</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G39" s="5">
         <v>2</v>
@@ -2721,7 +2721,7 @@
         <v>174</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
@@ -2754,7 +2754,7 @@
         <v>63</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G41" s="5">
         <v>2</v>
@@ -2787,7 +2787,7 @@
         <v>174</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G42" s="5">
         <v>2</v>
@@ -2820,7 +2820,7 @@
         <v>63</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G43" s="5">
         <v>2</v>
@@ -2853,7 +2853,7 @@
         <v>63</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G44" s="5">
         <v>2</v>
@@ -2886,7 +2886,7 @@
         <v>63</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G45" s="5">
         <v>2</v>
@@ -2919,7 +2919,7 @@
         <v>63</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G46" s="5">
         <v>2</v>
@@ -2952,7 +2952,7 @@
         <v>174</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G47" s="5">
         <v>2</v>
@@ -2985,7 +2985,7 @@
         <v>174</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G48" s="5">
         <v>2</v>
@@ -3018,7 +3018,7 @@
         <v>174</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G49" s="5">
         <v>2</v>
@@ -3051,7 +3051,7 @@
         <v>174</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G50" s="5">
         <v>2</v>
@@ -3084,7 +3084,7 @@
         <v>174</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G51" s="5">
         <v>2</v>
@@ -3117,7 +3117,7 @@
         <v>174</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G52" s="5">
         <v>2</v>

</xml_diff>